<commit_message>
feat: Integrate Audited Balance Sheet calculation engine and Excel download hub with live formula recalculation
</commit_message>
<xml_diff>
--- a/TMG_Key_Risk_Assessments_and_Weibull_Analysis.xlsx
+++ b/TMG_Key_Risk_Assessments_and_Weibull_Analysis.xlsx
@@ -18,6 +18,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Assesment(Labor &amp; Strife)" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weibull(Labor &amp; Strife)" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk score" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial statement" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source &amp; uses analysis" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Common size analysis" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ratios &amp; CFO Scorecard" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,11 +30,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -154,8 +159,61 @@
       <color rgb="0016A34A"/>
       <sz val="10.5"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00E0E7FF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001E293B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001E3A8A"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00047857"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B91C1C"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -228,8 +286,38 @@
         <bgColor rgb="00FEF2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E40AF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E293B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2E8F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE4E6"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="22">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -473,11 +561,25 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CBD5E1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00475569"/>
+      </top>
+      <bottom style="double">
+        <color rgb="001E293B"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -647,6 +749,93 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="24" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="24" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="15" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="28" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="24" fillId="16" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="24" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1037,6 +1226,12 @@
           <t>📌 أولاً: المفهوم الهندسي لإدارة المخاطر في المشروعات العملاقة (Megaprojects):</t>
         </is>
       </c>
+      <c r="B3" s="56" t="n"/>
+      <c r="C3" s="56" t="n"/>
+      <c r="D3" s="56" t="n"/>
+      <c r="E3" s="56" t="n"/>
+      <c r="F3" s="56" t="n"/>
+      <c r="G3" s="57" t="n"/>
     </row>
     <row r="4" ht="180" customHeight="1">
       <c r="A4" s="70" t="inlineStr">
@@ -1048,6 +1243,12 @@
 3. مين الخطر الأكبر اللي لو مخدناش بالنا منه فوراً، هيوقف الجداول الزمنية (Baseline Schedule) ويستنزف ميزانية المشروع (Cost Overrun)؟</t>
         </is>
       </c>
+      <c r="B4" s="56" t="n"/>
+      <c r="C4" s="56" t="n"/>
+      <c r="D4" s="56" t="n"/>
+      <c r="E4" s="56" t="n"/>
+      <c r="F4" s="56" t="n"/>
+      <c r="G4" s="57" t="n"/>
     </row>
     <row r="6" ht="26" customHeight="1">
       <c r="A6" s="71" t="inlineStr">
@@ -1055,6 +1256,12 @@
           <t>📑 ثانياً: الهيكل الإجرائي لصفحات الملف (Workflow Architecture):</t>
         </is>
       </c>
+      <c r="B6" s="56" t="n"/>
+      <c r="C6" s="56" t="n"/>
+      <c r="D6" s="56" t="n"/>
+      <c r="E6" s="56" t="n"/>
+      <c r="F6" s="56" t="n"/>
+      <c r="G6" s="57" t="n"/>
     </row>
     <row r="7" ht="216" customHeight="1">
       <c r="A7" s="72" t="inlineStr">
@@ -1066,6 +1273,12 @@
 4. مصفوفة الأولوية والترتيب النهائي (Risk score): حساب درجة الخطر الإجمالية (Risk Score = p × L) لترتيب الأولويات للمدير التنفيذي ومدير المشروع.</t>
         </is>
       </c>
+      <c r="B7" s="56" t="n"/>
+      <c r="C7" s="56" t="n"/>
+      <c r="D7" s="56" t="n"/>
+      <c r="E7" s="56" t="n"/>
+      <c r="F7" s="56" t="n"/>
+      <c r="G7" s="57" t="n"/>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="73" t="inlineStr">
@@ -1073,6 +1286,12 @@
           <t>📐 ثالثاً: الدليل الرياضي لمعادلات وايبول (Weibull Analysis Explained for Engineers):</t>
         </is>
       </c>
+      <c r="B9" s="56" t="n"/>
+      <c r="C9" s="56" t="n"/>
+      <c r="D9" s="56" t="n"/>
+      <c r="E9" s="56" t="n"/>
+      <c r="F9" s="56" t="n"/>
+      <c r="G9" s="57" t="n"/>
     </row>
     <row r="10" ht="270" customHeight="1">
       <c r="A10" s="74" t="inlineStr">
@@ -1085,6 +1304,12 @@
 • حدود التحكم عند مستوى ثقة 99% (Action Limit): ده السقف الحرج (Threshold). لو عدد المشاكل في أي أسبوع تجاوز هذا الرقم، يبقى النظام خرج عن السيطرة الإحصائية (Out-of-Control) ولازم تتدخل كمهندس فوراً وتصدر تقرير عدم مطابقة أو مذكرة للمدير العام.</t>
         </is>
       </c>
+      <c r="B10" s="56" t="n"/>
+      <c r="C10" s="56" t="n"/>
+      <c r="D10" s="56" t="n"/>
+      <c r="E10" s="56" t="n"/>
+      <c r="F10" s="56" t="n"/>
+      <c r="G10" s="57" t="n"/>
     </row>
     <row r="12" ht="26" customHeight="1">
       <c r="A12" s="75" t="inlineStr">
@@ -1092,6 +1317,12 @@
           <t>🏢 رابعاً: مصفوفة المخاطر الأربعة المدققة لمجموعة طلعت مصطفى (TMG Specific Risks):</t>
         </is>
       </c>
+      <c r="B12" s="56" t="n"/>
+      <c r="C12" s="56" t="n"/>
+      <c r="D12" s="56" t="n"/>
+      <c r="E12" s="56" t="n"/>
+      <c r="F12" s="56" t="n"/>
+      <c r="G12" s="57" t="n"/>
     </row>
     <row r="13" ht="342" customHeight="1">
       <c r="A13" s="76" t="inlineStr">
@@ -1106,6 +1337,12 @@
 مخاطر توقف العمالة بالمواقع الكبرى حال تعثر المقاول في سداد الأجور، وتستوجب تفعيل حساب وسيط (Escrow) لصرف مستحقات العمالة مباشرة.</t>
         </is>
       </c>
+      <c r="B13" s="56" t="n"/>
+      <c r="C13" s="56" t="n"/>
+      <c r="D13" s="56" t="n"/>
+      <c r="E13" s="56" t="n"/>
+      <c r="F13" s="56" t="n"/>
+      <c r="G13" s="57" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -1964,6 +2201,2586 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="79" t="inlineStr">
+        <is>
+          <t>Talaat Moustafa Group Holding (TMGH) — Audited Consolidated Financial Statements (2021 – 2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="80" t="inlineStr">
+        <is>
+          <t>Values in Thousands of Egyptian Pounds (EGP '000) — Sourced from EGX Audited Filings — Accounting Parity Checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="81" t="inlineStr">
+        <is>
+          <t>Line Item / البيان المحاسبي</t>
+        </is>
+      </c>
+      <c r="B3" s="82" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C3" s="82" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="D3" s="82" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E3" s="82" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="F3" s="82" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="G3" s="82" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="83" t="inlineStr">
+        <is>
+          <t>Sales Revenue (إيرادات النشاط الإجمالية)</t>
+        </is>
+      </c>
+      <c r="B4" s="84" t="inlineStr">
+        <is>
+          <t>REV_TOT</t>
+        </is>
+      </c>
+      <c r="C4" s="85" t="n">
+        <v>15357400</v>
+      </c>
+      <c r="D4" s="85" t="n">
+        <v>19870000</v>
+      </c>
+      <c r="E4" s="85" t="n">
+        <v>28430000</v>
+      </c>
+      <c r="F4" s="85" t="n">
+        <v>46900000</v>
+      </c>
+      <c r="G4" s="85" t="n">
+        <v>62500000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Cost of Goods Sold / Production (تكلفة الإيرادات)</t>
+        </is>
+      </c>
+      <c r="B5" s="87" t="inlineStr">
+        <is>
+          <t>COGS</t>
+        </is>
+      </c>
+      <c r="C5" s="88" t="n">
+        <v>-10287400</v>
+      </c>
+      <c r="D5" s="88" t="n">
+        <v>-13270000</v>
+      </c>
+      <c r="E5" s="88" t="n">
+        <v>-18960000</v>
+      </c>
+      <c r="F5" s="88" t="n">
+        <v>-31330000</v>
+      </c>
+      <c r="G5" s="88" t="n">
+        <v>-41620000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="83" t="inlineStr">
+        <is>
+          <t>Gross Profit (مجمل الربح)</t>
+        </is>
+      </c>
+      <c r="B6" s="84" t="inlineStr">
+        <is>
+          <t>GP</t>
+        </is>
+      </c>
+      <c r="C6" s="89">
+        <f>C4+C5</f>
+        <v/>
+      </c>
+      <c r="D6" s="89">
+        <f>D4+D5</f>
+        <v/>
+      </c>
+      <c r="E6" s="89">
+        <f>E4+E5</f>
+        <v/>
+      </c>
+      <c r="F6" s="89">
+        <f>F4+F5</f>
+        <v/>
+      </c>
+      <c r="G6" s="89">
+        <f>G4+G5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Selling, General &amp; Admin Expenses (مصروفات إدارية وعمومية)</t>
+        </is>
+      </c>
+      <c r="B7" s="87" t="inlineStr">
+        <is>
+          <t>SGA</t>
+        </is>
+      </c>
+      <c r="C7" s="88" t="n">
+        <v>-1380000</v>
+      </c>
+      <c r="D7" s="88" t="n">
+        <v>-1790000</v>
+      </c>
+      <c r="E7" s="88" t="n">
+        <v>-2560000</v>
+      </c>
+      <c r="F7" s="88" t="n">
+        <v>-4220000</v>
+      </c>
+      <c r="G7" s="88" t="n">
+        <v>-5620000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Depreciation &amp; Amortization (الإهلاك والاستهلاك)</t>
+        </is>
+      </c>
+      <c r="B8" s="87" t="inlineStr">
+        <is>
+          <t>DEP</t>
+        </is>
+      </c>
+      <c r="C8" s="88" t="n">
+        <v>-285000</v>
+      </c>
+      <c r="D8" s="88" t="n">
+        <v>-368000</v>
+      </c>
+      <c r="E8" s="88" t="n">
+        <v>-526000</v>
+      </c>
+      <c r="F8" s="88" t="n">
+        <v>-868000</v>
+      </c>
+      <c r="G8" s="88" t="n">
+        <v>-1160000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="83" t="inlineStr">
+        <is>
+          <t>Operating Profit / EBIT (أرباح التشغيل)</t>
+        </is>
+      </c>
+      <c r="B9" s="84" t="inlineStr">
+        <is>
+          <t>EBIT</t>
+        </is>
+      </c>
+      <c r="C9" s="89">
+        <f>C6+C7+C8</f>
+        <v/>
+      </c>
+      <c r="D9" s="89">
+        <f>D6+D7+D8</f>
+        <v/>
+      </c>
+      <c r="E9" s="89">
+        <f>E6+E7+E8</f>
+        <v/>
+      </c>
+      <c r="F9" s="89">
+        <f>F6+F7+F8</f>
+        <v/>
+      </c>
+      <c r="G9" s="89">
+        <f>G6+G7+G8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Finance Costs &amp; Interest (الأعباء التمويلية وفوائد الاقتراض)</t>
+        </is>
+      </c>
+      <c r="B10" s="87" t="inlineStr">
+        <is>
+          <t>FIN_EXP</t>
+        </is>
+      </c>
+      <c r="C10" s="88" t="n">
+        <v>-845000</v>
+      </c>
+      <c r="D10" s="88" t="n">
+        <v>-1190000</v>
+      </c>
+      <c r="E10" s="88" t="n">
+        <v>-1710000</v>
+      </c>
+      <c r="F10" s="88" t="n">
+        <v>-3280000</v>
+      </c>
+      <c r="G10" s="88" t="n">
+        <v>-4560000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + Investment Income &amp; Treasury (عوائد استثمارات وأذون)</t>
+        </is>
+      </c>
+      <c r="B11" s="87" t="inlineStr">
+        <is>
+          <t>INV_INC</t>
+        </is>
+      </c>
+      <c r="C11" s="88" t="n">
+        <v>210000</v>
+      </c>
+      <c r="D11" s="88" t="n">
+        <v>320000</v>
+      </c>
+      <c r="E11" s="88" t="n">
+        <v>480000</v>
+      </c>
+      <c r="F11" s="88" t="n">
+        <v>2450000</v>
+      </c>
+      <c r="G11" s="88" t="n">
+        <v>5200000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + FX Gains &amp; Other Income (أرباح فروق عملة ومكاسب أخرى)</t>
+        </is>
+      </c>
+      <c r="B12" s="87" t="inlineStr">
+        <is>
+          <t>FX_INC</t>
+        </is>
+      </c>
+      <c r="C12" s="88" t="n">
+        <v>15000</v>
+      </c>
+      <c r="D12" s="88" t="n">
+        <v>-25000</v>
+      </c>
+      <c r="E12" s="88" t="n">
+        <v>85000</v>
+      </c>
+      <c r="F12" s="88" t="n">
+        <v>3128000</v>
+      </c>
+      <c r="G12" s="88" t="n">
+        <v>9150000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="83" t="inlineStr">
+        <is>
+          <t>Earnings Before Tax / EBT (الأرباح قبل الضرائب)</t>
+        </is>
+      </c>
+      <c r="B13" s="84" t="inlineStr">
+        <is>
+          <t>EBT</t>
+        </is>
+      </c>
+      <c r="C13" s="89">
+        <f>C9+C10+C11+C12</f>
+        <v/>
+      </c>
+      <c r="D13" s="89">
+        <f>D9+D10+D11+D12</f>
+        <v/>
+      </c>
+      <c r="E13" s="89">
+        <f>E9+E10+E11+E12</f>
+        <v/>
+      </c>
+      <c r="F13" s="89">
+        <f>F9+F10+F11+F12</f>
+        <v/>
+      </c>
+      <c r="G13" s="89">
+        <f>G9+G10+G11+G12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Income Taxes (ضريبة الدخل المستحقة)</t>
+        </is>
+      </c>
+      <c r="B14" s="87" t="inlineStr">
+        <is>
+          <t>TAX</t>
+        </is>
+      </c>
+      <c r="C14" s="88" t="n">
+        <v>-1005000</v>
+      </c>
+      <c r="D14" s="88" t="n">
+        <v>-1317000</v>
+      </c>
+      <c r="E14" s="88" t="n">
+        <v>-1929000</v>
+      </c>
+      <c r="F14" s="88" t="n">
+        <v>-3660000</v>
+      </c>
+      <c r="G14" s="88" t="n">
+        <v>-5690000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="90" t="inlineStr">
+        <is>
+          <t>Net Profit After Taxes (صافي أرباح الفترة المجمعة)</t>
+        </is>
+      </c>
+      <c r="B15" s="91" t="inlineStr">
+        <is>
+          <t>NI_TOT</t>
+        </is>
+      </c>
+      <c r="C15" s="92">
+        <f>C13+C14</f>
+        <v/>
+      </c>
+      <c r="D15" s="92">
+        <f>D13+D14</f>
+        <v/>
+      </c>
+      <c r="E15" s="92">
+        <f>E13+E14</f>
+        <v/>
+      </c>
+      <c r="F15" s="92">
+        <f>F13+F14</f>
+        <v/>
+      </c>
+      <c r="G15" s="92">
+        <f>G13+G14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Attributable to Parent Company (نصيب مساهمي الشركة الأم)</t>
+        </is>
+      </c>
+      <c r="B16" s="87" t="inlineStr">
+        <is>
+          <t>PARENT_NI</t>
+        </is>
+      </c>
+      <c r="C16" s="88" t="n">
+        <v>1780000</v>
+      </c>
+      <c r="D16" s="88" t="n">
+        <v>2230000</v>
+      </c>
+      <c r="E16" s="88" t="n">
+        <v>3310000</v>
+      </c>
+      <c r="F16" s="88" t="n">
+        <v>7300000</v>
+      </c>
+      <c r="G16" s="88" t="n">
+        <v>14500000</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="86" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Attributable to Non-Controlling Interest (نصيب الحصص غير المسيطرة)</t>
+        </is>
+      </c>
+      <c r="B17" s="87" t="inlineStr">
+        <is>
+          <t>NCI_NI</t>
+        </is>
+      </c>
+      <c r="C17" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="88" t="n">
+        <v>1820000</v>
+      </c>
+      <c r="G17" s="88" t="n">
+        <v>3700000</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="93" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="94" t="inlineStr">
+        <is>
+          <t>ASSETS (الأصول)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="86" t="inlineStr">
+        <is>
+          <t>Cash and Cash Equivalents (النقدية وما في حكمها)</t>
+        </is>
+      </c>
+      <c r="B20" s="87" t="inlineStr">
+        <is>
+          <t>CASH</t>
+        </is>
+      </c>
+      <c r="C20" s="88" t="n">
+        <v>4210000</v>
+      </c>
+      <c r="D20" s="88" t="n">
+        <v>4780000</v>
+      </c>
+      <c r="E20" s="88" t="n">
+        <v>11500000</v>
+      </c>
+      <c r="F20" s="88" t="n">
+        <v>32000000</v>
+      </c>
+      <c r="G20" s="88" t="n">
+        <v>41200000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="86" t="inlineStr">
+        <is>
+          <t>Accounts and Notes Receivable (المدينون والعملاء وأوراق القبض)</t>
+        </is>
+      </c>
+      <c r="B21" s="87" t="inlineStr">
+        <is>
+          <t>REC</t>
+        </is>
+      </c>
+      <c r="C21" s="88" t="n">
+        <v>24500000</v>
+      </c>
+      <c r="D21" s="88" t="n">
+        <v>28600000</v>
+      </c>
+      <c r="E21" s="88" t="n">
+        <v>36400000</v>
+      </c>
+      <c r="F21" s="88" t="n">
+        <v>48200000</v>
+      </c>
+      <c r="G21" s="88" t="n">
+        <v>62800000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="86" t="inlineStr">
+        <is>
+          <t>Real Estate Work in Progress / Inventory (مشروعات قيد التنفيذ)</t>
+        </is>
+      </c>
+      <c r="B22" s="87" t="inlineStr">
+        <is>
+          <t>WIP</t>
+        </is>
+      </c>
+      <c r="C22" s="88" t="n">
+        <v>46800000</v>
+      </c>
+      <c r="D22" s="88" t="n">
+        <v>54200000</v>
+      </c>
+      <c r="E22" s="88" t="n">
+        <v>71300000</v>
+      </c>
+      <c r="F22" s="88" t="n">
+        <v>102500000</v>
+      </c>
+      <c r="G22" s="88" t="n">
+        <v>138500000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="86" t="inlineStr">
+        <is>
+          <t>Financial Investments at Fair Value (استثمارات مالية بالقيمة العادلة)</t>
+        </is>
+      </c>
+      <c r="B23" s="87" t="inlineStr">
+        <is>
+          <t>FIN_INV</t>
+        </is>
+      </c>
+      <c r="C23" s="88" t="n">
+        <v>1520500</v>
+      </c>
+      <c r="D23" s="88" t="n">
+        <v>2100200</v>
+      </c>
+      <c r="E23" s="88" t="n">
+        <v>4200000</v>
+      </c>
+      <c r="F23" s="88" t="n">
+        <v>8500000</v>
+      </c>
+      <c r="G23" s="88" t="n">
+        <v>14200000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="86" t="inlineStr">
+        <is>
+          <t>Fixed Assets &amp; CWIP Hotel Projects (أصول ثابتة ومشروعات فنادق)</t>
+        </is>
+      </c>
+      <c r="B24" s="87" t="inlineStr">
+        <is>
+          <t>FA_CWIP</t>
+        </is>
+      </c>
+      <c r="C24" s="88" t="n">
+        <v>31200000</v>
+      </c>
+      <c r="D24" s="88" t="n">
+        <v>36800000</v>
+      </c>
+      <c r="E24" s="88" t="n">
+        <v>51200000</v>
+      </c>
+      <c r="F24" s="88" t="n">
+        <v>81400000</v>
+      </c>
+      <c r="G24" s="88" t="n">
+        <v>107500000</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="86" t="inlineStr">
+        <is>
+          <t>Other Current &amp; Non-Current Assets (أصول أخرى)</t>
+        </is>
+      </c>
+      <c r="B25" s="87" t="inlineStr">
+        <is>
+          <t>OTH_AST</t>
+        </is>
+      </c>
+      <c r="C25" s="88" t="n">
+        <v>3470000</v>
+      </c>
+      <c r="D25" s="88" t="n">
+        <v>3920000</v>
+      </c>
+      <c r="E25" s="88" t="n">
+        <v>4620000</v>
+      </c>
+      <c r="F25" s="88" t="n">
+        <v>6200000</v>
+      </c>
+      <c r="G25" s="88" t="n">
+        <v>8000000</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="90" t="inlineStr">
+        <is>
+          <t>Total Assets (إجمالي الأصول المجمعة)</t>
+        </is>
+      </c>
+      <c r="B26" s="91" t="inlineStr">
+        <is>
+          <t>TOT_AST</t>
+        </is>
+      </c>
+      <c r="C26" s="92">
+        <f>SUM(C20:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="92">
+        <f>SUM(D20:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="92">
+        <f>SUM(E20:E25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="92">
+        <f>SUM(F20:F25)</f>
+        <v/>
+      </c>
+      <c r="G26" s="92">
+        <f>SUM(G20:G25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="93" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="94" t="inlineStr">
+        <is>
+          <t>LIABILITIES &amp; SHAREHOLDERS' EQUITY (الالتزامات وحقوق الملكية)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="86" t="inlineStr">
+        <is>
+          <t>Bank Overdrafts &amp; Short-term Credit Lines (تسهيلات بنكية قصيرة الأجل)</t>
+        </is>
+      </c>
+      <c r="B29" s="87" t="inlineStr">
+        <is>
+          <t>ST_LOANS</t>
+        </is>
+      </c>
+      <c r="C29" s="88" t="n">
+        <v>3800000</v>
+      </c>
+      <c r="D29" s="88" t="n">
+        <v>4500000</v>
+      </c>
+      <c r="E29" s="88" t="n">
+        <v>6200000</v>
+      </c>
+      <c r="F29" s="88" t="n">
+        <v>8900000</v>
+      </c>
+      <c r="G29" s="88" t="n">
+        <v>11200000</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="86" t="inlineStr">
+        <is>
+          <t>Trade and Notes Payable - Subcontractors (أوراق الدفع والمقاولين)</t>
+        </is>
+      </c>
+      <c r="B30" s="87" t="inlineStr">
+        <is>
+          <t>NOTES_PAY</t>
+        </is>
+      </c>
+      <c r="C30" s="88" t="n">
+        <v>5120000</v>
+      </c>
+      <c r="D30" s="88" t="n">
+        <v>7300000</v>
+      </c>
+      <c r="E30" s="88" t="n">
+        <v>9800000</v>
+      </c>
+      <c r="F30" s="88" t="n">
+        <v>13500000</v>
+      </c>
+      <c r="G30" s="88" t="n">
+        <v>15790000</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="86" t="inlineStr">
+        <is>
+          <t>Customer Advances &amp; Unearned Float (دفعات مقدمة من العملاء)</t>
+        </is>
+      </c>
+      <c r="B31" s="87" t="inlineStr">
+        <is>
+          <t>CUST_ADV</t>
+        </is>
+      </c>
+      <c r="C31" s="88" t="n">
+        <v>38500000</v>
+      </c>
+      <c r="D31" s="88" t="n">
+        <v>48200000</v>
+      </c>
+      <c r="E31" s="88" t="n">
+        <v>72000000</v>
+      </c>
+      <c r="F31" s="88" t="n">
+        <v>95000000</v>
+      </c>
+      <c r="G31" s="88" t="n">
+        <v>117680000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="86" t="inlineStr">
+        <is>
+          <t>Long-term Bank Debt (قروض بنكية وتسهيلات طويلة الأجل)</t>
+        </is>
+      </c>
+      <c r="B32" s="87" t="inlineStr">
+        <is>
+          <t>LT_DEBT</t>
+        </is>
+      </c>
+      <c r="C32" s="88" t="n">
+        <v>8200000</v>
+      </c>
+      <c r="D32" s="88" t="n">
+        <v>9800000</v>
+      </c>
+      <c r="E32" s="88" t="n">
+        <v>14500000</v>
+      </c>
+      <c r="F32" s="88" t="n">
+        <v>19800000</v>
+      </c>
+      <c r="G32" s="88" t="n">
+        <v>26500000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="86" t="inlineStr">
+        <is>
+          <t>Financial Lease Obligations - Off Balance (التزامات التأجير التمويلي)</t>
+        </is>
+      </c>
+      <c r="B33" s="87" t="inlineStr">
+        <is>
+          <t>LEASE_DEBT</t>
+        </is>
+      </c>
+      <c r="C33" s="88" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="D33" s="88" t="n">
+        <v>2100000</v>
+      </c>
+      <c r="E33" s="88" t="n">
+        <v>4800000</v>
+      </c>
+      <c r="F33" s="88" t="n">
+        <v>22100000</v>
+      </c>
+      <c r="G33" s="88" t="n">
+        <v>34400000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="86" t="inlineStr">
+        <is>
+          <t>Other Liabilities &amp; Provisions (التزامات ومخصصات أخرى)</t>
+        </is>
+      </c>
+      <c r="B34" s="87" t="inlineStr">
+        <is>
+          <t>OTH_LIAB</t>
+        </is>
+      </c>
+      <c r="C34" s="88" t="n">
+        <v>2140000</v>
+      </c>
+      <c r="D34" s="88" t="n">
+        <v>2600000</v>
+      </c>
+      <c r="E34" s="88" t="n">
+        <v>3630000</v>
+      </c>
+      <c r="F34" s="88" t="n">
+        <v>4730000</v>
+      </c>
+      <c r="G34" s="88" t="n">
+        <v>6830000</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="83" t="inlineStr">
+        <is>
+          <t>Total Liabilities (إجمالي الالتزامات)</t>
+        </is>
+      </c>
+      <c r="B35" s="84" t="inlineStr">
+        <is>
+          <t>TOT_LIAB</t>
+        </is>
+      </c>
+      <c r="C35" s="89">
+        <f>SUM(C29:C34)</f>
+        <v/>
+      </c>
+      <c r="D35" s="89">
+        <f>SUM(D29:D34)</f>
+        <v/>
+      </c>
+      <c r="E35" s="89">
+        <f>SUM(E29:E34)</f>
+        <v/>
+      </c>
+      <c r="F35" s="89">
+        <f>SUM(F29:F34)</f>
+        <v/>
+      </c>
+      <c r="G35" s="89">
+        <f>SUM(G29:G34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="93" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="86" t="inlineStr">
+        <is>
+          <t>Paid-in Share Capital (رأس المال المصدر والمدفوع)</t>
+        </is>
+      </c>
+      <c r="B37" s="87" t="inlineStr">
+        <is>
+          <t>CAPITAL</t>
+        </is>
+      </c>
+      <c r="C37" s="88" t="n">
+        <v>20635600</v>
+      </c>
+      <c r="D37" s="88" t="n">
+        <v>20635600</v>
+      </c>
+      <c r="E37" s="88" t="n">
+        <v>20635600</v>
+      </c>
+      <c r="F37" s="88" t="n">
+        <v>20635600</v>
+      </c>
+      <c r="G37" s="88" t="n">
+        <v>20635600</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="86" t="inlineStr">
+        <is>
+          <t>Legal &amp; General Reserves (احتياطيات وفروق ترجمة)</t>
+        </is>
+      </c>
+      <c r="B38" s="87" t="inlineStr">
+        <is>
+          <t>RESERVES</t>
+        </is>
+      </c>
+      <c r="C38" s="88" t="n">
+        <v>3450000</v>
+      </c>
+      <c r="D38" s="88" t="n">
+        <v>4100000</v>
+      </c>
+      <c r="E38" s="88" t="n">
+        <v>5200000</v>
+      </c>
+      <c r="F38" s="88" t="n">
+        <v>7800000</v>
+      </c>
+      <c r="G38" s="88" t="n">
+        <v>11500000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="86" t="inlineStr">
+        <is>
+          <t>Retained Earnings (أرباح مرحلة ومحتجزة)</t>
+        </is>
+      </c>
+      <c r="B39" s="87" t="inlineStr">
+        <is>
+          <t>RET_EARN</t>
+        </is>
+      </c>
+      <c r="C39" s="88" t="n">
+        <v>28654900</v>
+      </c>
+      <c r="D39" s="88" t="n">
+        <v>31164600</v>
+      </c>
+      <c r="E39" s="88" t="n">
+        <v>42454400</v>
+      </c>
+      <c r="F39" s="88" t="n">
+        <v>52834400</v>
+      </c>
+      <c r="G39" s="88" t="n">
+        <v>68164400</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="86" t="inlineStr">
+        <is>
+          <t>Non-Controlling Interests - ADQ ICON (الحصص غير المسيطرة)</t>
+        </is>
+      </c>
+      <c r="B40" s="87" t="inlineStr">
+        <is>
+          <t>NCI_EQ</t>
+        </is>
+      </c>
+      <c r="C40" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="88" t="n">
+        <v>33500000</v>
+      </c>
+      <c r="G40" s="88" t="n">
+        <v>59500000</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="83" t="inlineStr">
+        <is>
+          <t>Total Shareholders' Equity (إجمالي حقوق الملكية)</t>
+        </is>
+      </c>
+      <c r="B41" s="84" t="inlineStr">
+        <is>
+          <t>TOT_EQUITY</t>
+        </is>
+      </c>
+      <c r="C41" s="89">
+        <f>SUM(C37:C40)</f>
+        <v/>
+      </c>
+      <c r="D41" s="89">
+        <f>SUM(D37:D40)</f>
+        <v/>
+      </c>
+      <c r="E41" s="89">
+        <f>SUM(E37:E40)</f>
+        <v/>
+      </c>
+      <c r="F41" s="89">
+        <f>SUM(F37:F40)</f>
+        <v/>
+      </c>
+      <c r="G41" s="89">
+        <f>SUM(G37:G40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="90" t="inlineStr">
+        <is>
+          <t>Total Liabilities &amp; Equity (إجمالي الالتزامات وحقوق الملكية)</t>
+        </is>
+      </c>
+      <c r="B42" s="91" t="inlineStr">
+        <is>
+          <t>TOT_EQ_LIAB</t>
+        </is>
+      </c>
+      <c r="C42" s="92">
+        <f>C35+C41</f>
+        <v/>
+      </c>
+      <c r="D42" s="92">
+        <f>D35+D41</f>
+        <v/>
+      </c>
+      <c r="E42" s="92">
+        <f>E35+E41</f>
+        <v/>
+      </c>
+      <c r="F42" s="92">
+        <f>F35+F41</f>
+        <v/>
+      </c>
+      <c r="G42" s="92">
+        <f>G35+G41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="95" t="inlineStr">
+        <is>
+          <t>BALANCE CHECK: Assets - (Liab + Equity) (فحص التوازن)</t>
+        </is>
+      </c>
+      <c r="B43" s="96" t="inlineStr">
+        <is>
+          <t>CHECK</t>
+        </is>
+      </c>
+      <c r="C43" s="97">
+        <f>C26-C42</f>
+        <v/>
+      </c>
+      <c r="D43" s="97">
+        <f>D26-D42</f>
+        <v/>
+      </c>
+      <c r="E43" s="97">
+        <f>E26-E42</f>
+        <v/>
+      </c>
+      <c r="F43" s="97">
+        <f>F26-F42</f>
+        <v/>
+      </c>
+      <c r="G43" s="97">
+        <f>G26-G42</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A28:G28"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="98" t="inlineStr">
+        <is>
+          <t>Talaat Moustafa Group Holding — Source &amp; Uses Analysis (FY2024 vs FY2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="99" t="inlineStr">
+        <is>
+          <t>Tracking Balance Sheet Dynamic Shifts &amp; Liquidity Deployment (Values in EGP '000)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="100" t="inlineStr">
+        <is>
+          <t>Balance Sheet Line Item / بند الميزانية</t>
+        </is>
+      </c>
+      <c r="B3" s="101" t="inlineStr">
+        <is>
+          <t>At Dec 31, 2024</t>
+        </is>
+      </c>
+      <c r="C3" s="101" t="inlineStr">
+        <is>
+          <t>At Dec 31, 2025</t>
+        </is>
+      </c>
+      <c r="D3" s="101" t="inlineStr">
+        <is>
+          <t>Change (التغير)</t>
+        </is>
+      </c>
+      <c r="E3" s="101" t="inlineStr">
+        <is>
+          <t>Source (مصدر نقد)</t>
+        </is>
+      </c>
+      <c r="F3" s="101" t="inlineStr">
+        <is>
+          <t>Use (استخدام سيولة)</t>
+        </is>
+      </c>
+      <c r="G3" s="101" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="86" t="inlineStr">
+        <is>
+          <t>Cash and Cash Equivalents (نقدية وما في حكمها)</t>
+        </is>
+      </c>
+      <c r="B4" s="88">
+        <f>'Financial statement'!F20</f>
+        <v/>
+      </c>
+      <c r="C4" s="88">
+        <f>'Financial statement'!G20</f>
+        <v/>
+      </c>
+      <c r="D4" s="88">
+        <f>C4-B4</f>
+        <v/>
+      </c>
+      <c r="E4" s="88">
+        <f>IF(D4&lt;0, -D4, 0)</f>
+        <v/>
+      </c>
+      <c r="F4" s="88">
+        <f>IF(D4&gt;0, D4, 0)</f>
+        <v/>
+      </c>
+      <c r="G4" s="84">
+        <f>IF(E4&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="86" t="inlineStr">
+        <is>
+          <t>Accounts and Notes Receivable (المدينون وأوراق القبض)</t>
+        </is>
+      </c>
+      <c r="B5" s="88">
+        <f>'Financial statement'!F21</f>
+        <v/>
+      </c>
+      <c r="C5" s="88">
+        <f>'Financial statement'!G21</f>
+        <v/>
+      </c>
+      <c r="D5" s="88">
+        <f>C5-B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="88">
+        <f>IF(D5&lt;0, -D5, 0)</f>
+        <v/>
+      </c>
+      <c r="F5" s="88">
+        <f>IF(D5&gt;0, D5, 0)</f>
+        <v/>
+      </c>
+      <c r="G5" s="84">
+        <f>IF(E5&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="86" t="inlineStr">
+        <is>
+          <t>Real Estate Work in Progress (مشروعات قيد التنفيذ)</t>
+        </is>
+      </c>
+      <c r="B6" s="88">
+        <f>'Financial statement'!F22</f>
+        <v/>
+      </c>
+      <c r="C6" s="88">
+        <f>'Financial statement'!G22</f>
+        <v/>
+      </c>
+      <c r="D6" s="88">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="88">
+        <f>IF(D6&lt;0, -D6, 0)</f>
+        <v/>
+      </c>
+      <c r="F6" s="88">
+        <f>IF(D6&gt;0, D6, 0)</f>
+        <v/>
+      </c>
+      <c r="G6" s="84">
+        <f>IF(E6&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="86" t="inlineStr">
+        <is>
+          <t>Financial Investments (استثمارات مالية وأذون)</t>
+        </is>
+      </c>
+      <c r="B7" s="88">
+        <f>'Financial statement'!F23</f>
+        <v/>
+      </c>
+      <c r="C7" s="88">
+        <f>'Financial statement'!G23</f>
+        <v/>
+      </c>
+      <c r="D7" s="88">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="88">
+        <f>IF(D7&lt;0, -D7, 0)</f>
+        <v/>
+      </c>
+      <c r="F7" s="88">
+        <f>IF(D7&gt;0, D7, 0)</f>
+        <v/>
+      </c>
+      <c r="G7" s="84">
+        <f>IF(E7&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="86" t="inlineStr">
+        <is>
+          <t>Fixed Assets &amp; CWIP (أصول ثابتة ومشروعات فنادق)</t>
+        </is>
+      </c>
+      <c r="B8" s="88">
+        <f>'Financial statement'!F24</f>
+        <v/>
+      </c>
+      <c r="C8" s="88">
+        <f>'Financial statement'!G24</f>
+        <v/>
+      </c>
+      <c r="D8" s="88">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="88">
+        <f>IF(D8&lt;0, -D8, 0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="88">
+        <f>IF(D8&gt;0, D8, 0)</f>
+        <v/>
+      </c>
+      <c r="G8" s="84">
+        <f>IF(E8&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="86" t="inlineStr">
+        <is>
+          <t>Other Assets (أصول أخرى)</t>
+        </is>
+      </c>
+      <c r="B9" s="88">
+        <f>'Financial statement'!F25</f>
+        <v/>
+      </c>
+      <c r="C9" s="88">
+        <f>'Financial statement'!G25</f>
+        <v/>
+      </c>
+      <c r="D9" s="88">
+        <f>C9-B9</f>
+        <v/>
+      </c>
+      <c r="E9" s="88">
+        <f>IF(D9&lt;0, -D9, 0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="88">
+        <f>IF(D9&gt;0, D9, 0)</f>
+        <v/>
+      </c>
+      <c r="G9" s="84">
+        <f>IF(E9&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="86" t="inlineStr">
+        <is>
+          <t>Bank Overdrafts &amp; Short-term Credit Lines (تسهيلات بنكية)</t>
+        </is>
+      </c>
+      <c r="B10" s="88">
+        <f>'Financial statement'!F29</f>
+        <v/>
+      </c>
+      <c r="C10" s="88">
+        <f>'Financial statement'!G29</f>
+        <v/>
+      </c>
+      <c r="D10" s="88">
+        <f>C10-B10</f>
+        <v/>
+      </c>
+      <c r="E10" s="88">
+        <f>IF(D10&gt;0, D10, 0)</f>
+        <v/>
+      </c>
+      <c r="F10" s="88">
+        <f>IF(D10&lt;0, -D10, 0)</f>
+        <v/>
+      </c>
+      <c r="G10" s="84">
+        <f>IF(E10&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="86" t="inlineStr">
+        <is>
+          <t>Trade and Notes Payable (أوراق دفع ومقاولين)</t>
+        </is>
+      </c>
+      <c r="B11" s="88">
+        <f>'Financial statement'!F30</f>
+        <v/>
+      </c>
+      <c r="C11" s="88">
+        <f>'Financial statement'!G30</f>
+        <v/>
+      </c>
+      <c r="D11" s="88">
+        <f>C11-B11</f>
+        <v/>
+      </c>
+      <c r="E11" s="88">
+        <f>IF(D11&gt;0, D11, 0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="88">
+        <f>IF(D11&lt;0, -D11, 0)</f>
+        <v/>
+      </c>
+      <c r="G11" s="84">
+        <f>IF(E11&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="86" t="inlineStr">
+        <is>
+          <t>Customer Advances (دفعات مقدمة من العملاء)</t>
+        </is>
+      </c>
+      <c r="B12" s="88">
+        <f>'Financial statement'!F31</f>
+        <v/>
+      </c>
+      <c r="C12" s="88">
+        <f>'Financial statement'!G31</f>
+        <v/>
+      </c>
+      <c r="D12" s="88">
+        <f>C12-B12</f>
+        <v/>
+      </c>
+      <c r="E12" s="88">
+        <f>IF(D12&gt;0, D12, 0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="88">
+        <f>IF(D12&lt;0, -D12, 0)</f>
+        <v/>
+      </c>
+      <c r="G12" s="84">
+        <f>IF(E12&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="86" t="inlineStr">
+        <is>
+          <t>Long-term Bank Debt (قروض بنكية طويلة الأجل)</t>
+        </is>
+      </c>
+      <c r="B13" s="88">
+        <f>'Financial statement'!F32</f>
+        <v/>
+      </c>
+      <c r="C13" s="88">
+        <f>'Financial statement'!G32</f>
+        <v/>
+      </c>
+      <c r="D13" s="88">
+        <f>C13-B13</f>
+        <v/>
+      </c>
+      <c r="E13" s="88">
+        <f>IF(D13&gt;0, D13, 0)</f>
+        <v/>
+      </c>
+      <c r="F13" s="88">
+        <f>IF(D13&lt;0, -D13, 0)</f>
+        <v/>
+      </c>
+      <c r="G13" s="84">
+        <f>IF(E13&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="86" t="inlineStr">
+        <is>
+          <t>Financial Lease Obligations (التزامات التأجير التمويلي)</t>
+        </is>
+      </c>
+      <c r="B14" s="88">
+        <f>'Financial statement'!F33</f>
+        <v/>
+      </c>
+      <c r="C14" s="88">
+        <f>'Financial statement'!G33</f>
+        <v/>
+      </c>
+      <c r="D14" s="88">
+        <f>C14-B14</f>
+        <v/>
+      </c>
+      <c r="E14" s="88">
+        <f>IF(D14&gt;0, D14, 0)</f>
+        <v/>
+      </c>
+      <c r="F14" s="88">
+        <f>IF(D14&lt;0, -D14, 0)</f>
+        <v/>
+      </c>
+      <c r="G14" s="84">
+        <f>IF(E14&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="86" t="inlineStr">
+        <is>
+          <t>Other Liabilities &amp; Provisions (التزامات ومخصصات أخرى)</t>
+        </is>
+      </c>
+      <c r="B15" s="88">
+        <f>'Financial statement'!F34</f>
+        <v/>
+      </c>
+      <c r="C15" s="88">
+        <f>'Financial statement'!G34</f>
+        <v/>
+      </c>
+      <c r="D15" s="88">
+        <f>C15-B15</f>
+        <v/>
+      </c>
+      <c r="E15" s="88">
+        <f>IF(D15&gt;0, D15, 0)</f>
+        <v/>
+      </c>
+      <c r="F15" s="88">
+        <f>IF(D15&lt;0, -D15, 0)</f>
+        <v/>
+      </c>
+      <c r="G15" s="84">
+        <f>IF(E15&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="86" t="inlineStr">
+        <is>
+          <t>Share Capital (رأس المال المصدر)</t>
+        </is>
+      </c>
+      <c r="B16" s="88">
+        <f>'Financial statement'!F37</f>
+        <v/>
+      </c>
+      <c r="C16" s="88">
+        <f>'Financial statement'!G37</f>
+        <v/>
+      </c>
+      <c r="D16" s="88">
+        <f>C16-B16</f>
+        <v/>
+      </c>
+      <c r="E16" s="88">
+        <f>IF(D16&gt;0, D16, 0)</f>
+        <v/>
+      </c>
+      <c r="F16" s="88">
+        <f>IF(D16&lt;0, -D16, 0)</f>
+        <v/>
+      </c>
+      <c r="G16" s="84">
+        <f>IF(E16&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="86" t="inlineStr">
+        <is>
+          <t>Reserves &amp; Translation Differences (احتياطيات وفروق ترجمة)</t>
+        </is>
+      </c>
+      <c r="B17" s="88">
+        <f>'Financial statement'!F38</f>
+        <v/>
+      </c>
+      <c r="C17" s="88">
+        <f>'Financial statement'!G38</f>
+        <v/>
+      </c>
+      <c r="D17" s="88">
+        <f>C17-B17</f>
+        <v/>
+      </c>
+      <c r="E17" s="88">
+        <f>IF(D17&gt;0, D17, 0)</f>
+        <v/>
+      </c>
+      <c r="F17" s="88">
+        <f>IF(D17&lt;0, -D17, 0)</f>
+        <v/>
+      </c>
+      <c r="G17" s="84">
+        <f>IF(E17&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="86" t="inlineStr">
+        <is>
+          <t>Retained Earnings (أرباح مرحلة محتجزة)</t>
+        </is>
+      </c>
+      <c r="B18" s="88">
+        <f>'Financial statement'!F39</f>
+        <v/>
+      </c>
+      <c r="C18" s="88">
+        <f>'Financial statement'!G39</f>
+        <v/>
+      </c>
+      <c r="D18" s="88">
+        <f>C18-B18</f>
+        <v/>
+      </c>
+      <c r="E18" s="88">
+        <f>IF(D18&gt;0, D18, 0)</f>
+        <v/>
+      </c>
+      <c r="F18" s="88">
+        <f>IF(D18&lt;0, -D18, 0)</f>
+        <v/>
+      </c>
+      <c r="G18" s="84">
+        <f>IF(E18&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="86" t="inlineStr">
+        <is>
+          <t>Non-Controlling Interests / ADQ ICON (حصص غير مسيطرة)</t>
+        </is>
+      </c>
+      <c r="B19" s="88">
+        <f>'Financial statement'!F40</f>
+        <v/>
+      </c>
+      <c r="C19" s="88">
+        <f>'Financial statement'!G40</f>
+        <v/>
+      </c>
+      <c r="D19" s="88">
+        <f>C19-B19</f>
+        <v/>
+      </c>
+      <c r="E19" s="88">
+        <f>IF(D19&gt;0, D19, 0)</f>
+        <v/>
+      </c>
+      <c r="F19" s="88">
+        <f>IF(D19&lt;0, -D19, 0)</f>
+        <v/>
+      </c>
+      <c r="G19" s="84">
+        <f>IF(E19&gt;0, "Source (مصدر)", "Use (استخدام)")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="102" t="inlineStr">
+        <is>
+          <t>Total Sources &amp; Uses (إجمالي مصادر واستخدامات الأموال)</t>
+        </is>
+      </c>
+      <c r="B20" s="103" t="n"/>
+      <c r="C20" s="103" t="n"/>
+      <c r="D20" s="103" t="n"/>
+      <c r="E20" s="104">
+        <f>SUM(E4:E19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="104">
+        <f>SUM(F4:F19)</f>
+        <v/>
+      </c>
+      <c r="G20" s="105">
+        <f>IF(E20=F20, "Balanced ✓ (توازن تام)", "Variance")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="79" t="inlineStr">
+        <is>
+          <t>Talaat Moustafa Group Holding — Vertical Common Size Analysis (FY2023 – FY2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="80" t="inlineStr">
+        <is>
+          <t>Income Statement as % of Total Sales &amp; Balance Sheet as % of Total Assets</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="81" t="inlineStr">
+        <is>
+          <t>Statement Line Item / البند المحاسبي</t>
+        </is>
+      </c>
+      <c r="B3" s="82" t="inlineStr">
+        <is>
+          <t>FY2023 (EGP '000)</t>
+        </is>
+      </c>
+      <c r="C3" s="82" t="inlineStr">
+        <is>
+          <t>% of Base (2023)</t>
+        </is>
+      </c>
+      <c r="D3" s="82" t="inlineStr">
+        <is>
+          <t>FY2024 (EGP '000)</t>
+        </is>
+      </c>
+      <c r="E3" s="82" t="inlineStr">
+        <is>
+          <t>% of Base (2024)</t>
+        </is>
+      </c>
+      <c r="F3" s="82" t="inlineStr">
+        <is>
+          <t>FY2025 (EGP '000)</t>
+        </is>
+      </c>
+      <c r="G3" s="82" t="inlineStr">
+        <is>
+          <t>% of Base (2025)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="83" t="inlineStr">
+        <is>
+          <t>Sales Revenue (إجمالي الإيرادات)</t>
+        </is>
+      </c>
+      <c r="B4" s="106">
+        <f>'Financial statement'!E4</f>
+        <v/>
+      </c>
+      <c r="C4" s="107">
+        <f>B4/$B$4</f>
+        <v/>
+      </c>
+      <c r="D4" s="106">
+        <f>'Financial statement'!F4</f>
+        <v/>
+      </c>
+      <c r="E4" s="107">
+        <f>D4/$D$4</f>
+        <v/>
+      </c>
+      <c r="F4" s="106">
+        <f>'Financial statement'!G4</f>
+        <v/>
+      </c>
+      <c r="G4" s="107">
+        <f>F4/$F$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="86" t="inlineStr">
+        <is>
+          <t>Cost of Goods Sold (تكلفة الإيرادات)</t>
+        </is>
+      </c>
+      <c r="B5" s="88">
+        <f>'Financial statement'!E5</f>
+        <v/>
+      </c>
+      <c r="C5" s="108">
+        <f>B5/$B$4</f>
+        <v/>
+      </c>
+      <c r="D5" s="88">
+        <f>'Financial statement'!F5</f>
+        <v/>
+      </c>
+      <c r="E5" s="108">
+        <f>D5/$D$4</f>
+        <v/>
+      </c>
+      <c r="F5" s="88">
+        <f>'Financial statement'!G5</f>
+        <v/>
+      </c>
+      <c r="G5" s="108">
+        <f>F5/$F$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="83" t="inlineStr">
+        <is>
+          <t>Gross Profit (مجمل الربح)</t>
+        </is>
+      </c>
+      <c r="B6" s="106">
+        <f>'Financial statement'!E6</f>
+        <v/>
+      </c>
+      <c r="C6" s="107">
+        <f>B6/$B$4</f>
+        <v/>
+      </c>
+      <c r="D6" s="106">
+        <f>'Financial statement'!F6</f>
+        <v/>
+      </c>
+      <c r="E6" s="107">
+        <f>D6/$D$4</f>
+        <v/>
+      </c>
+      <c r="F6" s="106">
+        <f>'Financial statement'!G6</f>
+        <v/>
+      </c>
+      <c r="G6" s="107">
+        <f>F6/$F$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="86" t="inlineStr">
+        <is>
+          <t>Selling, General &amp; Admin (مصروفات إدارية وعمومية)</t>
+        </is>
+      </c>
+      <c r="B7" s="88">
+        <f>'Financial statement'!E7</f>
+        <v/>
+      </c>
+      <c r="C7" s="108">
+        <f>B7/$B$4</f>
+        <v/>
+      </c>
+      <c r="D7" s="88">
+        <f>'Financial statement'!F7</f>
+        <v/>
+      </c>
+      <c r="E7" s="108">
+        <f>D7/$D$4</f>
+        <v/>
+      </c>
+      <c r="F7" s="88">
+        <f>'Financial statement'!G7</f>
+        <v/>
+      </c>
+      <c r="G7" s="108">
+        <f>F7/$F$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="83" t="inlineStr">
+        <is>
+          <t>Operating Profit / EBIT (أرباح التشغيل)</t>
+        </is>
+      </c>
+      <c r="B8" s="106">
+        <f>'Financial statement'!E9</f>
+        <v/>
+      </c>
+      <c r="C8" s="107">
+        <f>B8/$B$4</f>
+        <v/>
+      </c>
+      <c r="D8" s="106">
+        <f>'Financial statement'!F9</f>
+        <v/>
+      </c>
+      <c r="E8" s="107">
+        <f>D8/$D$4</f>
+        <v/>
+      </c>
+      <c r="F8" s="106">
+        <f>'Financial statement'!G9</f>
+        <v/>
+      </c>
+      <c r="G8" s="107">
+        <f>F8/$F$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="86" t="inlineStr">
+        <is>
+          <t>Finance Costs / Interest (الأعباء التمويلية)</t>
+        </is>
+      </c>
+      <c r="B9" s="88">
+        <f>'Financial statement'!E10</f>
+        <v/>
+      </c>
+      <c r="C9" s="108">
+        <f>B9/$B$4</f>
+        <v/>
+      </c>
+      <c r="D9" s="88">
+        <f>'Financial statement'!F10</f>
+        <v/>
+      </c>
+      <c r="E9" s="108">
+        <f>D9/$D$4</f>
+        <v/>
+      </c>
+      <c r="F9" s="88">
+        <f>'Financial statement'!G10</f>
+        <v/>
+      </c>
+      <c r="G9" s="108">
+        <f>F9/$F$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="83" t="inlineStr">
+        <is>
+          <t>Net Profit After Taxes (صافي الربح المجمع)</t>
+        </is>
+      </c>
+      <c r="B10" s="106">
+        <f>'Financial statement'!E15</f>
+        <v/>
+      </c>
+      <c r="C10" s="107">
+        <f>B10/$B$4</f>
+        <v/>
+      </c>
+      <c r="D10" s="106">
+        <f>'Financial statement'!F15</f>
+        <v/>
+      </c>
+      <c r="E10" s="107">
+        <f>D10/$D$4</f>
+        <v/>
+      </c>
+      <c r="F10" s="106">
+        <f>'Financial statement'!G15</f>
+        <v/>
+      </c>
+      <c r="G10" s="107">
+        <f>F10/$F$4</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="98" t="inlineStr">
+        <is>
+          <t>Talaat Moustafa Group Holding — Construction CFO Strategic Ratio Scorecard (FY21 – FY25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="99" t="inlineStr">
+        <is>
+          <t>Audited Forensic Metrics: Liquidity, Working Capital Cycles, Off-Balance Leases &amp; Subcontractor Exposure</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="100" t="inlineStr">
+        <is>
+          <t>Metric / Ratio Classification</t>
+        </is>
+      </c>
+      <c r="B3" s="101" t="inlineStr">
+        <is>
+          <t>Target Norm</t>
+        </is>
+      </c>
+      <c r="C3" s="101" t="inlineStr">
+        <is>
+          <t>FY2021</t>
+        </is>
+      </c>
+      <c r="D3" s="101" t="inlineStr">
+        <is>
+          <t>FY2022</t>
+        </is>
+      </c>
+      <c r="E3" s="101" t="inlineStr">
+        <is>
+          <t>FY2023</t>
+        </is>
+      </c>
+      <c r="F3" s="101" t="inlineStr">
+        <is>
+          <t>FY2024</t>
+        </is>
+      </c>
+      <c r="G3" s="101" t="inlineStr">
+        <is>
+          <t>FY2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="83" t="inlineStr">
+        <is>
+          <t>Current Ratio (النسبة الجارية)</t>
+        </is>
+      </c>
+      <c r="B4" s="87" t="inlineStr">
+        <is>
+          <t>1.2x - 1.5x</t>
+        </is>
+      </c>
+      <c r="C4" s="109" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="D4" s="109" t="inlineStr">
+        <is>
+          <t>1.58</t>
+        </is>
+      </c>
+      <c r="E4" s="109" t="inlineStr">
+        <is>
+          <t>1.49</t>
+        </is>
+      </c>
+      <c r="F4" s="109" t="inlineStr">
+        <is>
+          <t>1.54</t>
+        </is>
+      </c>
+      <c r="G4" s="109" t="inlineStr">
+        <is>
+          <t>1.63</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="83" t="inlineStr">
+        <is>
+          <t>Quick Ratio (Acid-Test بدون مخزون)</t>
+        </is>
+      </c>
+      <c r="B5" s="87" t="inlineStr">
+        <is>
+          <t>&gt; 0.8x</t>
+        </is>
+      </c>
+      <c r="C5" s="109" t="inlineStr">
+        <is>
+          <t>0.60</t>
+        </is>
+      </c>
+      <c r="D5" s="109" t="inlineStr">
+        <is>
+          <t>0.54</t>
+        </is>
+      </c>
+      <c r="E5" s="109" t="inlineStr">
+        <is>
+          <t>0.57</t>
+        </is>
+      </c>
+      <c r="F5" s="109" t="inlineStr">
+        <is>
+          <t>0.67</t>
+        </is>
+      </c>
+      <c r="G5" s="109" t="inlineStr">
+        <is>
+          <t>0.73</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="83" t="inlineStr">
+        <is>
+          <t>Cash Ratio (نسبة النقدية الفورية)</t>
+        </is>
+      </c>
+      <c r="B6" s="87" t="inlineStr">
+        <is>
+          <t>&gt; 0.2x</t>
+        </is>
+      </c>
+      <c r="C6" s="109" t="inlineStr">
+        <is>
+          <t>0.09</t>
+        </is>
+      </c>
+      <c r="D6" s="109" t="inlineStr">
+        <is>
+          <t>0.08</t>
+        </is>
+      </c>
+      <c r="E6" s="109" t="inlineStr">
+        <is>
+          <t>0.13</t>
+        </is>
+      </c>
+      <c r="F6" s="109" t="inlineStr">
+        <is>
+          <t>0.27</t>
+        </is>
+      </c>
+      <c r="G6" s="109" t="inlineStr">
+        <is>
+          <t>0.28</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="83" t="inlineStr">
+        <is>
+          <t>Days Payable Outstanding - DPO (فترة سداد الموردين)</t>
+        </is>
+      </c>
+      <c r="B7" s="87" t="inlineStr">
+        <is>
+          <t>60-90 days</t>
+        </is>
+      </c>
+      <c r="C7" s="110" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D7" s="110" t="inlineStr">
+        <is>
+          <t>134 days</t>
+        </is>
+      </c>
+      <c r="E7" s="110" t="inlineStr">
+        <is>
+          <t>141 days</t>
+        </is>
+      </c>
+      <c r="F7" s="110" t="inlineStr">
+        <is>
+          <t>138 days</t>
+        </is>
+      </c>
+      <c r="G7" s="110" t="inlineStr">
+        <is>
+          <t>160 days</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="83" t="inlineStr">
+        <is>
+          <t>Days Sales Inventory - DSI (فترة دوران المخزون)</t>
+        </is>
+      </c>
+      <c r="B8" s="87" t="inlineStr">
+        <is>
+          <t>360-720d</t>
+        </is>
+      </c>
+      <c r="C8" s="109" t="inlineStr">
+        <is>
+          <t>1,659d</t>
+        </is>
+      </c>
+      <c r="D8" s="109" t="inlineStr">
+        <is>
+          <t>1,490d</t>
+        </is>
+      </c>
+      <c r="E8" s="109" t="inlineStr">
+        <is>
+          <t>1,372d</t>
+        </is>
+      </c>
+      <c r="F8" s="109" t="inlineStr">
+        <is>
+          <t>1,194d</t>
+        </is>
+      </c>
+      <c r="G8" s="109" t="inlineStr">
+        <is>
+          <t>1,214d</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="83" t="inlineStr">
+        <is>
+          <t>Days Sales Outstanding - DSO (فترة تحصيل العملاء)</t>
+        </is>
+      </c>
+      <c r="B9" s="87" t="inlineStr">
+        <is>
+          <t>90-180d</t>
+        </is>
+      </c>
+      <c r="C9" s="109" t="inlineStr">
+        <is>
+          <t>582d</t>
+        </is>
+      </c>
+      <c r="D9" s="109" t="inlineStr">
+        <is>
+          <t>525d</t>
+        </is>
+      </c>
+      <c r="E9" s="109" t="inlineStr">
+        <is>
+          <t>467d</t>
+        </is>
+      </c>
+      <c r="F9" s="109" t="inlineStr">
+        <is>
+          <t>375d</t>
+        </is>
+      </c>
+      <c r="G9" s="109" t="inlineStr">
+        <is>
+          <t>367d</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="83" t="inlineStr">
+        <is>
+          <t>Cash Conversion Cycle - CCC (دورة التحويل النقدي)</t>
+        </is>
+      </c>
+      <c r="B10" s="87" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C10" s="109" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D10" s="109" t="inlineStr">
+        <is>
+          <t>1,881d</t>
+        </is>
+      </c>
+      <c r="E10" s="109" t="inlineStr">
+        <is>
+          <t>1,698d</t>
+        </is>
+      </c>
+      <c r="F10" s="109" t="inlineStr">
+        <is>
+          <t>1,431d</t>
+        </is>
+      </c>
+      <c r="G10" s="109" t="inlineStr">
+        <is>
+          <t>1,421d</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="83" t="inlineStr">
+        <is>
+          <t>Debt to Equity Ratio (الدين إلى الملكية)</t>
+        </is>
+      </c>
+      <c r="B11" s="87" t="inlineStr">
+        <is>
+          <t>&lt; 1.5x</t>
+        </is>
+      </c>
+      <c r="C11" s="109" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
+      </c>
+      <c r="D11" s="109" t="inlineStr">
+        <is>
+          <t>1.33</t>
+        </is>
+      </c>
+      <c r="E11" s="109" t="inlineStr">
+        <is>
+          <t>1.62</t>
+        </is>
+      </c>
+      <c r="F11" s="109" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="G11" s="109" t="inlineStr">
+        <is>
+          <t>1.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="83" t="inlineStr">
+        <is>
+          <t>Interest Coverage Ratio - ICR (تغطية الفوائد)</t>
+        </is>
+      </c>
+      <c r="B12" s="87" t="inlineStr">
+        <is>
+          <t>&gt; 3.0x</t>
+        </is>
+      </c>
+      <c r="C12" s="110" t="inlineStr">
+        <is>
+          <t>4.02x</t>
+        </is>
+      </c>
+      <c r="D12" s="110" t="inlineStr">
+        <is>
+          <t>3.73x</t>
+        </is>
+      </c>
+      <c r="E12" s="110" t="inlineStr">
+        <is>
+          <t>3.74x</t>
+        </is>
+      </c>
+      <c r="F12" s="110" t="inlineStr">
+        <is>
+          <t>3.20x</t>
+        </is>
+      </c>
+      <c r="G12" s="110" t="inlineStr">
+        <is>
+          <t>3.09x</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="83" t="inlineStr">
+        <is>
+          <t>Off-Balance Financial Leases (التأجير التمويلي)</t>
+        </is>
+      </c>
+      <c r="B13" s="87" t="inlineStr">
+        <is>
+          <t>Minimal</t>
+        </is>
+      </c>
+      <c r="C13" s="110" t="inlineStr">
+        <is>
+          <t>1.20 B</t>
+        </is>
+      </c>
+      <c r="D13" s="110" t="inlineStr">
+        <is>
+          <t>2.10 B</t>
+        </is>
+      </c>
+      <c r="E13" s="110" t="inlineStr">
+        <is>
+          <t>4.80 B</t>
+        </is>
+      </c>
+      <c r="F13" s="110" t="inlineStr">
+        <is>
+          <t>22.10 B</t>
+        </is>
+      </c>
+      <c r="G13" s="110" t="inlineStr">
+        <is>
+          <t>34.40 B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="83" t="inlineStr">
+        <is>
+          <t>Gross Profit Margin (هامش مجمل الربح)</t>
+        </is>
+      </c>
+      <c r="B14" s="87" t="inlineStr">
+        <is>
+          <t>&gt; 30%</t>
+        </is>
+      </c>
+      <c r="C14" s="111" t="inlineStr">
+        <is>
+          <t>33.0%</t>
+        </is>
+      </c>
+      <c r="D14" s="111" t="inlineStr">
+        <is>
+          <t>33.2%</t>
+        </is>
+      </c>
+      <c r="E14" s="111" t="inlineStr">
+        <is>
+          <t>33.3%</t>
+        </is>
+      </c>
+      <c r="F14" s="111" t="inlineStr">
+        <is>
+          <t>33.2%</t>
+        </is>
+      </c>
+      <c r="G14" s="111" t="inlineStr">
+        <is>
+          <t>33.4%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="83" t="inlineStr">
+        <is>
+          <t>Net Profit Margin (هامش صافي الربح)</t>
+        </is>
+      </c>
+      <c r="B15" s="87" t="inlineStr">
+        <is>
+          <t>&gt; 15%</t>
+        </is>
+      </c>
+      <c r="C15" s="111" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+      <c r="D15" s="111" t="inlineStr">
+        <is>
+          <t>11.2%</t>
+        </is>
+      </c>
+      <c r="E15" s="111" t="inlineStr">
+        <is>
+          <t>11.6%</t>
+        </is>
+      </c>
+      <c r="F15" s="111" t="inlineStr">
+        <is>
+          <t>19.4%</t>
+        </is>
+      </c>
+      <c r="G15" s="111" t="inlineStr">
+        <is>
+          <t>29.1%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="83" t="inlineStr">
+        <is>
+          <t>Return on Equity - ROE (العائد على الملكية)</t>
+        </is>
+      </c>
+      <c r="B16" s="87" t="inlineStr">
+        <is>
+          <t>&gt; 10%</t>
+        </is>
+      </c>
+      <c r="C16" s="111" t="inlineStr">
+        <is>
+          <t>3.37%</t>
+        </is>
+      </c>
+      <c r="D16" s="111" t="inlineStr">
+        <is>
+          <t>3.99%</t>
+        </is>
+      </c>
+      <c r="E16" s="111" t="inlineStr">
+        <is>
+          <t>4.85%</t>
+        </is>
+      </c>
+      <c r="F16" s="111" t="inlineStr">
+        <is>
+          <t>7.95%</t>
+        </is>
+      </c>
+      <c r="G16" s="111" t="inlineStr">
+        <is>
+          <t>11.39%</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="83" t="inlineStr">
+        <is>
+          <t>Return on Assets - ROA (العائد على الأصول)</t>
+        </is>
+      </c>
+      <c r="B17" s="87" t="inlineStr">
+        <is>
+          <t>&gt; 3%</t>
+        </is>
+      </c>
+      <c r="C17" s="111" t="inlineStr">
+        <is>
+          <t>1.59%</t>
+        </is>
+      </c>
+      <c r="D17" s="111" t="inlineStr">
+        <is>
+          <t>1.71%</t>
+        </is>
+      </c>
+      <c r="E17" s="111" t="inlineStr">
+        <is>
+          <t>1.85%</t>
+        </is>
+      </c>
+      <c r="F17" s="111" t="inlineStr">
+        <is>
+          <t>3.27%</t>
+        </is>
+      </c>
+      <c r="G17" s="111" t="inlineStr">
+        <is>
+          <t>4.89%</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2171,7 +4988,7 @@
       <c r="F10" s="59" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="60" t="n"/>
+      <c r="A11" s="63" t="n"/>
       <c r="B11" s="61" t="n"/>
       <c r="C11" s="61" t="n"/>
       <c r="D11" s="61" t="n"/>

</xml_diff>